<commit_message>
Upload remaining operational data artifacts
</commit_message>
<xml_diff>
--- a/data/processed/modeling/aceptacion_digital_redes_medios_sentimiento_semanal.xlsx
+++ b/data/processed/modeling/aceptacion_digital_redes_medios_sentimiento_semanal.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sentimiento_semanal" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sentimiento_semanal'!$A$1:$I$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sentimiento_semanal'!$A$1:$I$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,16 +21,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -50,7 +47,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -58,21 +55,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -439,14 +428,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
@@ -2838,7 +2827,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.5072463768115942</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>0.2</v>
@@ -2847,13 +2836,13 @@
         <v>-0.2289023717595146</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.1009353369037931</v>
+        <v>0.02716856483114054</v>
       </c>
       <c r="H77" s="2" t="n">
         <v>0.1528107680126682</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0.1268730524582307</v>
+        <v>0.0899896664219044</v>
       </c>
     </row>
     <row r="78">
@@ -2869,7 +2858,7 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>0.6231884057971014</v>
+        <v>0.6842105263157895</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>0.09677419354838709</v>
@@ -2878,13 +2867,13 @@
         <v>-0.122060470324748</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.1052090920574953</v>
+        <v>0.1211586643975283</v>
       </c>
       <c r="H78" s="2" t="n">
         <v>0.1413802016024813</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>0.1232946468299883</v>
+        <v>0.1312694330000048</v>
       </c>
     </row>
     <row r="79">
@@ -2900,7 +2889,7 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>0.75</v>
+        <v>0.7281553398058253</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>0.4188034188034188</v>
@@ -2909,13 +2898,13 @@
         <v>-0.4370477568740955</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.0002473960639255284</v>
+        <v>-0.005462221777095377</v>
       </c>
       <c r="H79" s="2" t="n">
         <v>0.07403651115618662</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>0.03714195361005607</v>
+        <v>0.03428714468954562</v>
       </c>
     </row>
     <row r="80">
@@ -2931,7 +2920,7 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>0.7878787878787878</v>
+        <v>0.6859504132231405</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>0.286624203821656</v>
@@ -2940,17 +2929,141 @@
         <v>-0.262483994878361</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.09355609798026393</v>
+        <v>0.06691471004989276</v>
       </c>
       <c r="H80" s="2" t="n">
         <v>0.1218498311249675</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>0.1077029645526157</v>
+        <v>0.09438227058743015</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B81" t="n">
+        <v>15</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2026-W15</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>0.7864077669902912</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>-0.2191235059760956</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>0.110472470964671</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>0.1378848728246319</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>0.1241786718946514</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B82" t="n">
+        <v>16</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-W16</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>0.6880733944954128</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>0.2380952380952381</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>-0.2512820512820513</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>0.06687791935569266</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0.07456</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>0.07071895967784633</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B83" t="n">
+        <v>17</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2026-W17</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>0.6883116883116883</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>0.04035874439461883</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>-0.2435703479576399</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>0.04214202741675304</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>0.009624958513109858</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>0.02588349296493145</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B84" t="n">
+        <v>18</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2026-W18</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>-0.1587301587301587</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>0.0732244276596991</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>0.1154303847679492</v>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>0.09432740621382416</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I80"/>
+  <autoFilter ref="A1:I84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>